<commit_message>
Correcao nos codigos dos testes de alocacao para rodar testes com qualquer quantidade de beneficiarios
</commit_message>
<xml_diff>
--- a/alocacao/saidas_1500/resumo_custos.xlsx
+++ b/alocacao/saidas_1500/resumo_custos.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados_Custos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados_Custos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -427,78 +439,78 @@
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="114" customWidth="1" min="10" max="10"/>
-    <col width="117" customWidth="1" min="11" max="11"/>
+    <col width="90" customWidth="1" min="10" max="10"/>
+    <col width="93" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nome da Instância</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Total de Entregas</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Pico de Abastecimento (Max/Dia)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Custo Modelo Exato (M1)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Custo Modelo Anual (M2)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Custo Heurística</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Gap Heurística vs M1 (%)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Gap M2 vs M1 (%)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caminho da Entrada</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Pasta de Saída</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>abastecimento_00_1550</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>7488</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>294</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>abastecimento_full_1500</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>7852</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>300</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -512,26 +524,26 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_1500\abastecimento_00_1550.csv</t>
+          <t>/home/guilherme/ModelsAndHeristics/alocacao/entradas_1500/abastecimento_full_1500.csv</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1500\alocacao_abastecimento_00_1550</t>
+          <t>/home/guilherme/ModelsAndHeristics/alocacao/saidas_1500/alocacao_abastecimento_full_1500</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>abastecimento_10wlim_1500</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>7567</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>88</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>abastecimento_limite_1500</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>7553</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>259</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -545,26 +557,26 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_1500\abastecimento_10wlim_1500.csv</t>
+          <t>/home/guilherme/ModelsAndHeristics/alocacao/entradas_1500/abastecimento_limite_1500.csv</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1500\alocacao_abastecimento_10wlim_1500</t>
+          <t>/home/guilherme/ModelsAndHeristics/alocacao/saidas_1500/alocacao_abastecimento_limite_1500</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>abastecimento_full_1500</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>7852</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>300</v>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>abastecimento_10wlim_1500</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>7567</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>88</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -578,26 +590,26 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_1500\abastecimento_full_1500.csv</t>
+          <t>/home/guilherme/ModelsAndHeristics/alocacao/entradas_1500/abastecimento_10wlim_1500.csv</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1500\alocacao_abastecimento_full_1500</t>
+          <t>/home/guilherme/ModelsAndHeristics/alocacao/saidas_1500/alocacao_abastecimento_10wlim_1500</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>abastecimento_limite_1500</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>7553</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>259</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1500</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7488</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>294</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -611,12 +623,12 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_1500\abastecimento_limite_1500.csv</t>
+          <t>/home/guilherme/ModelsAndHeristics/alocacao/entradas_1500/abastecimento_00_1500.csv</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1500\alocacao_abastecimento_limite_1500</t>
+          <t>/home/guilherme/ModelsAndHeristics/alocacao/saidas_1500/alocacao_abastecimento_00_1500</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Resultados testes de alocacao 1500
</commit_message>
<xml_diff>
--- a/alocacao/saidas_1500/resumo_custos.xlsx
+++ b/alocacao/saidas_1500/resumo_custos.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados_Custos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resultados_Custos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,23 +42,16 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,202 +423,242 @@
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="90" customWidth="1" min="10" max="10"/>
-    <col width="93" customWidth="1" min="11" max="11"/>
+    <col width="114" customWidth="1" min="10" max="10"/>
+    <col width="117" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Nome da Instância</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Total de Entregas</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Pico de Abastecimento (Max/Dia)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Custo Modelo Exato (M1)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Custo Modelo Anual (M2)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Custo Heurística</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Gap Heurística vs M1 (%)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Gap M2 vs M1 (%)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Caminho da Entrada</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Pasta de Saída</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>abastecimento_full_1500</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>7852</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>300</v>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1500</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>7488</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>294</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Erro Execução</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>256337.18</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>258909.82</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>340833.62</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>/home/guilherme/ModelsAndHeristics/alocacao/entradas_1500/abastecimento_full_1500.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_1500\abastecimento_00_1500.csv</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>/home/guilherme/ModelsAndHeristics/alocacao/saidas_1500/alocacao_abastecimento_full_1500</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1500\alocacao_abastecimento_00_1500</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>abastecimento_limite_1500</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>7553</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>259</v>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>abastecimento_10wlim_1500</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>7567</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>88</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Erro Execução</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>256254.89</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>256696.36</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>333075.77</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.17</v>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>/home/guilherme/ModelsAndHeristics/alocacao/entradas_1500/abastecimento_limite_1500.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_1500\abastecimento_10wlim_1500.csv</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>/home/guilherme/ModelsAndHeristics/alocacao/saidas_1500/alocacao_abastecimento_limite_1500</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1500\alocacao_abastecimento_10wlim_1500</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>abastecimento_10wlim_1500</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>7567</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>88</v>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>abastecimento_full_1500</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>7852</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>300</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Erro Execução</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>268644.83</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>273550.73</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>362412.22</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>1.83</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>/home/guilherme/ModelsAndHeristics/alocacao/entradas_1500/abastecimento_10wlim_1500.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_1500\abastecimento_full_1500.csv</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>/home/guilherme/ModelsAndHeristics/alocacao/saidas_1500/alocacao_abastecimento_10wlim_1500</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1500\alocacao_abastecimento_full_1500</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>abastecimento_00_1500</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>7488</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>294</v>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>abastecimento_limite_1500</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>7553</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>259</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Erro Execução</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+          <t>Sucesso</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>257300.14</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>261185.68</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>346701.64</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>34.75</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>1.51</v>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>/home/guilherme/ModelsAndHeristics/alocacao/entradas_1500/abastecimento_00_1500.csv</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas_1500\abastecimento_limite_1500.csv</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>/home/guilherme/ModelsAndHeristics/alocacao/saidas_1500/alocacao_abastecimento_00_1500</t>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1500\alocacao_abastecimento_limite_1500</t>
         </is>
       </c>
     </row>

</xml_diff>